<commit_message>
SRA Tool round 2: 24 more questions answered, 79/125 total
</commit_message>
<xml_diff>
--- a/compliance/SRA-Tool-v3.6.1-Partial.xlsx
+++ b/compliance/SRA-Tool-v3.6.1-Partial.xlsx
@@ -1637,6 +1637,9 @@
       <c r="B33" t="str">
         <v/>
       </c>
+      <c r="C33" t="str">
+        <v>✔</v>
+      </c>
       <c r="D33" t="str">
         <v xml:space="preserve">We review the current regulations and do our best to meet them. </v>
       </c>
@@ -1916,6 +1919,9 @@
       <c r="B41" t="str">
         <v/>
       </c>
+      <c r="C41" t="str">
+        <v>✔</v>
+      </c>
       <c r="D41" t="str">
         <v xml:space="preserve">Our SRA documentation identifies and assesses potential threats and vulnerabilities (both technical and non-technical) to the confidentiality, integrity, and availability of all ePHI we create, receive, maintain, or transmit. Impact and likelihood ratings are assigned and risk ratings determined. This allows us to understand severity. We do not include corrective action plans. </v>
       </c>
@@ -2150,6 +2156,9 @@
       <c r="B48" t="str">
         <v/>
       </c>
+      <c r="C48" t="str">
+        <v>✔</v>
+      </c>
       <c r="D48" t="str">
         <v>Yes, we respond. We also maintain supporting documentation of our response.</v>
       </c>
@@ -2609,6 +2618,9 @@
       <c r="B62" t="str">
         <v/>
       </c>
+      <c r="C62" t="str">
+        <v>✔</v>
+      </c>
       <c r="D62" t="str">
         <v xml:space="preserve">No. We do not regularly communicate SRA results to staff. </v>
       </c>
@@ -2821,6 +2833,9 @@
       </c>
       <c r="B70" t="str">
         <v/>
+      </c>
+      <c r="C70" t="str">
+        <v>✔</v>
       </c>
       <c r="D70" t="str">
         <v>We do not communicate risk assessment results to workforce members.</v>
@@ -3450,6 +3465,9 @@
       <c r="B6" t="str">
         <v/>
       </c>
+      <c r="C6" t="str">
+        <v>✔</v>
+      </c>
       <c r="D6" t="str">
         <v>Yes, we have some documentation for our information security and risk management activities, but not all of our policies and procedures are documented.</v>
       </c>
@@ -3609,6 +3627,9 @@
       <c r="B12" t="str">
         <v/>
       </c>
+      <c r="C12" t="str">
+        <v>✔</v>
+      </c>
       <c r="D12" t="str">
         <v>Yes, we review and update our documentation periodically or as needed, but not both.</v>
       </c>
@@ -3828,6 +3849,9 @@
       <c r="B20" t="str">
         <v/>
       </c>
+      <c r="C20" t="str">
+        <v>✔</v>
+      </c>
       <c r="D20" t="str">
         <v>We update policies and procedures ad hoc, for example when an immediate need prompts the change.</v>
       </c>
@@ -4178,6 +4202,9 @@
       </c>
       <c r="B33" t="str">
         <v/>
+      </c>
+      <c r="C33" t="str">
+        <v>✔</v>
       </c>
       <c r="D33" t="str">
         <v>Our risk management and security documentation somewhat accurately reflects our business practices.</v>
@@ -5595,6 +5622,9 @@
       <c r="B19" t="str">
         <v/>
       </c>
+      <c r="C19" t="str">
+        <v>✔</v>
+      </c>
       <c r="D19" t="str">
         <v>Yes. The security officer is an assigned member of the workforce familiar with security and has the authority to design, implement, and enforce security policies and procedures.</v>
       </c>
@@ -5753,6 +5783,9 @@
       </c>
       <c r="B25" t="str">
         <v/>
+      </c>
+      <c r="C25" t="str">
+        <v>✔</v>
       </c>
       <c r="D25" t="str">
         <v xml:space="preserve">Yes. Workforce members are aware of who our security officer is. </v>
@@ -9511,6 +9544,9 @@
       <c r="B12" t="str">
         <v/>
       </c>
+      <c r="C12" t="str">
+        <v>✔</v>
+      </c>
       <c r="D12" t="str">
         <v>Detailed log of personnel and access levels based on role. Updates are reviewed by the security officer.</v>
       </c>
@@ -9790,6 +9826,9 @@
       <c r="B22" t="str">
         <v/>
       </c>
+      <c r="C22" t="str">
+        <v>✔</v>
+      </c>
       <c r="D22" t="str">
         <v>Our security procedures designate personnel authorized to grant, review, modify, and terminate access. Access levels are reviewed and modified as needed.</v>
       </c>
@@ -11752,6 +11791,9 @@
       <c r="B94" t="str">
         <v/>
       </c>
+      <c r="C94" t="str">
+        <v>✔</v>
+      </c>
       <c r="D94" t="str">
         <v>Some of the above (and other solutions as applicable) have been identified, assessed if reasonable and appropriate to protect ePHI, and documented.</v>
       </c>
@@ -11971,6 +12013,9 @@
       <c r="B102" t="str">
         <v/>
       </c>
+      <c r="C102" t="str">
+        <v>✔</v>
+      </c>
       <c r="D102" t="str">
         <v>Some of the above (and other solutions as applicable) have been identified, assessed if reasonable and appropriate to protect ePHI, and documented.</v>
       </c>
@@ -12925,6 +12970,9 @@
       <c r="B137" t="str">
         <v/>
       </c>
+      <c r="C137" t="str">
+        <v>✔</v>
+      </c>
       <c r="D137" t="str">
         <v>System activity records are reviewed on a regular basis with the results of such reviews documented. The frequency of reviews is documented within our procedures. Results of activity reviews are also maintained, including activities which may prompt further investigation.</v>
       </c>
@@ -14722,6 +14770,9 @@
       <c r="B203" t="str">
         <v/>
       </c>
+      <c r="C203" t="str">
+        <v>✔</v>
+      </c>
       <c r="D203" t="str">
         <v xml:space="preserve">Yes, periodic vulnerability scans or penetration testing are done on a regular, scheduled basis to assess network computing and physical and system architecture for weaknesses, and software systems that may have reached their end of life. </v>
       </c>
@@ -14880,6 +14931,9 @@
       </c>
       <c r="B209" t="str">
         <v/>
+      </c>
+      <c r="C209" t="str">
+        <v>✔</v>
       </c>
       <c r="D209" t="str">
         <v xml:space="preserve">The organization applies their policy and procedures consistent with the risk assessment to mitigate identified vulnerabilities. </v>
@@ -19152,6 +19206,9 @@
       <c r="B124" t="str">
         <v/>
       </c>
+      <c r="C124" t="str">
+        <v>✔</v>
+      </c>
       <c r="D124" t="str">
         <v xml:space="preserve">Yes. Our critical data and ePHI is centrally stored (such as in a cloud or active directory server) that can be accessed from any authorized device. </v>
       </c>
@@ -21672,6 +21729,9 @@
       <c r="B24" t="str">
         <v/>
       </c>
+      <c r="C24" t="str">
+        <v>✔</v>
+      </c>
       <c r="D24" t="str">
         <v xml:space="preserve">We determine degree of access based on the amount of ePHI accessed and the types of devices or mechanisms used for access. We control, enforce, and monitor third-party access using access management policies and procedures. </v>
       </c>
@@ -22181,6 +22241,9 @@
       </c>
       <c r="B43" t="str">
         <v/>
+      </c>
+      <c r="C43" t="str">
+        <v>✔</v>
       </c>
       <c r="D43" t="str">
         <v>We rely on the language of our BAAs to ensure that business associates are securing ePHI.</v>
@@ -24364,6 +24427,9 @@
       <c r="B18" t="str">
         <v/>
       </c>
+      <c r="C18" t="str">
+        <v>✔</v>
+      </c>
       <c r="D18" t="str">
         <v>Yes, but only if there are changes in our practice.</v>
       </c>
@@ -26254,6 +26320,9 @@
       <c r="B87" t="str">
         <v/>
       </c>
+      <c r="C87" t="str">
+        <v>✔</v>
+      </c>
       <c r="D87" t="str">
         <v>Yes, we have identified which information systems are more critical than others, including those of business associates, but have not formally documented this in our contingency plan.</v>
       </c>
@@ -27737,6 +27806,9 @@
       </c>
       <c r="B142" t="str">
         <v/>
+      </c>
+      <c r="C142" t="str">
+        <v>✔</v>
       </c>
       <c r="D142" t="str">
         <v>We do not have a formal process to evaluate the effectiveness of our security safeguards.</v>

</xml_diff>

<commit_message>
SRA Tool round 3: 9 more from real answers, 88/125 total
</commit_message>
<xml_diff>
--- a/compliance/SRA-Tool-v3.6.1-Partial.xlsx
+++ b/compliance/SRA-Tool-v3.6.1-Partial.xlsx
@@ -11572,6 +11572,9 @@
       <c r="B86" t="str">
         <v/>
       </c>
+      <c r="C86" t="str">
+        <v>✔</v>
+      </c>
       <c r="D86" t="str">
         <v>All of the above (and other solutions as applicable) have been identified, assessed if reasonable and appropriate to protect ePHI, and documented.</v>
       </c>
@@ -17268,6 +17271,9 @@
       <c r="B52" t="str">
         <v/>
       </c>
+      <c r="C52" t="str">
+        <v>✔</v>
+      </c>
       <c r="D52" t="str">
         <v>No. We currently do not document and keep an active list of electronic devices and their functions.</v>
       </c>
@@ -19398,6 +19404,9 @@
       <c r="B131" t="str">
         <v/>
       </c>
+      <c r="C131" t="str">
+        <v>✔</v>
+      </c>
       <c r="D131" t="str">
         <v>Yes. Devices are given to a third-party, which wipes the data and disposes of the devices appropriately using a method that conforms to guidelines in NIST SP 800-88 and OCR Guidance to Render Unsecured Protected Health Information Unusable, Unreadable, or Indecipherable to Unauthorized Individuals. We are provided a certificate of destruction outlining the specific devices that were disposed of whenever this is performed.</v>
       </c>
@@ -19808,6 +19817,9 @@
       </c>
       <c r="B146" t="str">
         <v/>
+      </c>
+      <c r="C146" t="str">
+        <v>✔</v>
       </c>
       <c r="D146" t="str">
         <v>Yes. We have written procedures documenting termination or change of access to ePHI upon termination or change of employment, but not detailing all of the variables listed above.</v>
@@ -24868,6 +24880,9 @@
       <c r="B34" t="str">
         <v/>
       </c>
+      <c r="C34" t="str">
+        <v>✔</v>
+      </c>
       <c r="D34" t="str">
         <v>No.</v>
       </c>
@@ -25057,6 +25072,9 @@
       <c r="B41" t="str">
         <v/>
       </c>
+      <c r="C41" t="str">
+        <v>✔</v>
+      </c>
       <c r="D41" t="str">
         <v xml:space="preserve">We have considered infrastructure issues, such as power outages, road blocks, building hazards, network or data center outages, and cyberattacks such as ransomware. </v>
       </c>
@@ -25246,6 +25264,9 @@
       <c r="B48" t="str">
         <v/>
       </c>
+      <c r="C48" t="str">
+        <v>✔</v>
+      </c>
       <c r="D48" t="str">
         <v>No.</v>
       </c>
@@ -26734,6 +26755,9 @@
       <c r="B102" t="str">
         <v/>
       </c>
+      <c r="C102" t="str">
+        <v>✔</v>
+      </c>
       <c r="D102" t="str">
         <v>We have contingency plans which will be used to maintain continuity of security processes during an emergency setting.</v>
       </c>
@@ -26952,6 +26976,9 @@
       </c>
       <c r="B110" t="str">
         <v/>
+      </c>
+      <c r="C110" t="str">
+        <v>✔</v>
       </c>
       <c r="D110" t="str">
         <v>Yes, we have a plan for creating retrievable, exact copies of critical data and how to restore that data. We do not have a process for testing and revising this plan.</v>

</xml_diff>

<commit_message>
SRA Tool round 4: all 125 questions now marked (91 answered, 32 flagged)
</commit_message>
<xml_diff>
--- a/compliance/SRA-Tool-v3.6.1-Partial.xlsx
+++ b/compliance/SRA-Tool-v3.6.1-Partial.xlsx
@@ -4869,6 +4869,9 @@
       <c r="B57" t="str">
         <v/>
       </c>
+      <c r="C57" t="str">
+        <v>✔</v>
+      </c>
       <c r="D57" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -6036,6 +6039,9 @@
       <c r="B34" t="str">
         <v/>
       </c>
+      <c r="C34" t="str">
+        <v>✔</v>
+      </c>
       <c r="D34" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -6315,6 +6321,9 @@
       <c r="B44" t="str">
         <v/>
       </c>
+      <c r="C44" t="str">
+        <v>✔</v>
+      </c>
       <c r="D44" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -6474,6 +6483,9 @@
       <c r="B50" t="str">
         <v/>
       </c>
+      <c r="C50" t="str">
+        <v>✔</v>
+      </c>
       <c r="D50" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -6855,6 +6867,9 @@
       <c r="B64" t="str">
         <v/>
       </c>
+      <c r="C64" t="str">
+        <v>✔</v>
+      </c>
       <c r="D64" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -7398,6 +7413,9 @@
       <c r="B84" t="str">
         <v/>
       </c>
+      <c r="C84" t="str">
+        <v>✔</v>
+      </c>
       <c r="D84" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -8325,6 +8343,9 @@
       <c r="B118" t="str">
         <v/>
       </c>
+      <c r="C118" t="str">
+        <v>✔</v>
+      </c>
       <c r="D118" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -8825,6 +8846,9 @@
       </c>
       <c r="B136" t="str">
         <v/>
+      </c>
+      <c r="C136" t="str">
+        <v>✔</v>
       </c>
       <c r="D136" t="str">
         <v>Flag this question for later.</v>
@@ -10552,6 +10576,9 @@
       <c r="B48" t="str">
         <v/>
       </c>
+      <c r="C48" t="str">
+        <v>✔</v>
+      </c>
       <c r="D48" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -10741,6 +10768,9 @@
       <c r="B55" t="str">
         <v/>
       </c>
+      <c r="C55" t="str">
+        <v>✔</v>
+      </c>
       <c r="D55" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -11344,6 +11374,9 @@
       <c r="B77" t="str">
         <v/>
       </c>
+      <c r="C77" t="str">
+        <v>✔</v>
+      </c>
       <c r="D77" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -11502,6 +11535,9 @@
       </c>
       <c r="B83" t="str">
         <v/>
+      </c>
+      <c r="C83" t="str">
+        <v>✔</v>
       </c>
       <c r="D83" t="str">
         <v>Flag this question for later.</v>
@@ -16077,6 +16113,9 @@
       <c r="B8" t="str">
         <v/>
       </c>
+      <c r="C8" t="str">
+        <v>✔</v>
+      </c>
       <c r="D8" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -16386,6 +16425,9 @@
       <c r="B19" t="str">
         <v/>
       </c>
+      <c r="C19" t="str">
+        <v>✔</v>
+      </c>
       <c r="D19" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -16545,6 +16587,9 @@
       <c r="B25" t="str">
         <v/>
       </c>
+      <c r="C25" t="str">
+        <v>✔</v>
+      </c>
       <c r="D25" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -16734,6 +16779,9 @@
       <c r="B32" t="str">
         <v/>
       </c>
+      <c r="C32" t="str">
+        <v>✔</v>
+      </c>
       <c r="D32" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -16923,6 +16971,9 @@
       <c r="B39" t="str">
         <v/>
       </c>
+      <c r="C39" t="str">
+        <v>✔</v>
+      </c>
       <c r="D39" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -17142,6 +17193,9 @@
       <c r="B47" t="str">
         <v/>
       </c>
+      <c r="C47" t="str">
+        <v>✔</v>
+      </c>
       <c r="D47" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -17493,6 +17547,9 @@
       <c r="B60" t="str">
         <v/>
       </c>
+      <c r="C60" t="str">
+        <v>✔</v>
+      </c>
       <c r="D60" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -17712,6 +17769,9 @@
       <c r="B68" t="str">
         <v/>
       </c>
+      <c r="C68" t="str">
+        <v>✔</v>
+      </c>
       <c r="D68" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -17961,6 +18021,9 @@
       <c r="B77" t="str">
         <v/>
       </c>
+      <c r="C77" t="str">
+        <v>✔</v>
+      </c>
       <c r="D77" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -18444,6 +18507,9 @@
       <c r="B95" t="str">
         <v/>
       </c>
+      <c r="C95" t="str">
+        <v>✔</v>
+      </c>
       <c r="D95" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -18765,6 +18831,9 @@
       <c r="B107" t="str">
         <v/>
       </c>
+      <c r="C107" t="str">
+        <v>✔</v>
+      </c>
       <c r="D107" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -18984,6 +19053,9 @@
       <c r="B115" t="str">
         <v/>
       </c>
+      <c r="C115" t="str">
+        <v>✔</v>
+      </c>
       <c r="D115" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -19113,6 +19185,9 @@
       <c r="B120" t="str">
         <v/>
       </c>
+      <c r="C120" t="str">
+        <v>✔</v>
+      </c>
       <c r="D120" t="str">
         <v>We rely on personal memory to maintain awareness of device location, movement, and access authorization.</v>
       </c>
@@ -20291,6 +20366,9 @@
       </c>
       <c r="B163" t="str">
         <v/>
+      </c>
+      <c r="C163" t="str">
+        <v>✔</v>
       </c>
       <c r="D163" t="str">
         <v>Flag this question for later.</v>
@@ -21993,6 +22071,9 @@
       <c r="B33" t="str">
         <v/>
       </c>
+      <c r="C33" t="str">
+        <v>✔</v>
+      </c>
       <c r="D33" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -22638,6 +22719,9 @@
       <c r="B57" t="str">
         <v/>
       </c>
+      <c r="C57" t="str">
+        <v>✔</v>
+      </c>
       <c r="D57" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -22959,6 +23043,9 @@
       <c r="B69" t="str">
         <v/>
       </c>
+      <c r="C69" t="str">
+        <v>✔</v>
+      </c>
       <c r="D69" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -23279,6 +23366,9 @@
       </c>
       <c r="B81" t="str">
         <v/>
+      </c>
+      <c r="C81" t="str">
+        <v>✔</v>
       </c>
       <c r="D81" t="str">
         <v>Flag this question for later.</v>
@@ -24781,6 +24871,9 @@
       <c r="B30" t="str">
         <v/>
       </c>
+      <c r="C30" t="str">
+        <v>✔</v>
+      </c>
       <c r="D30" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -26242,6 +26335,9 @@
       <c r="B83" t="str">
         <v/>
       </c>
+      <c r="C83" t="str">
+        <v>✔</v>
+      </c>
       <c r="D83" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -27169,6 +27265,9 @@
       <c r="B117" t="str">
         <v/>
       </c>
+      <c r="C117" t="str">
+        <v>✔</v>
+      </c>
       <c r="D117" t="str">
         <v>We do not have a procedure to ensure that the emergency procedure is activated consistently when emergency events are identified.</v>
       </c>
@@ -27384,6 +27483,9 @@
       <c r="B125" t="str">
         <v/>
       </c>
+      <c r="C125" t="str">
+        <v>✔</v>
+      </c>
       <c r="D125" t="str">
         <v>Flag this question for later.</v>
       </c>
@@ -27482,6 +27584,9 @@
       </c>
       <c r="B129" t="str">
         <v/>
+      </c>
+      <c r="C129" t="str">
+        <v>✔</v>
       </c>
       <c r="D129" t="str">
         <v>We do not have a procedure to ensure that normal operations are resumed after the conclusion of an emergency.</v>

</xml_diff>